<commit_message>
Add 28 blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 214
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-adventures.report.xlsx
+++ b/tools/importer/reports/import-adventures.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="226">
   <si>
     <t>_reportFile</t>
   </si>
@@ -43,22 +43,40 @@
     <t>url</t>
   </si>
   <si>
+    <t>about.report.json</t>
+  </si>
+  <si>
+    <t>["hero-adventure","cards-article","cards-promo","columns-story","tabs-team"]</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>about</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>adventures</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:58:09.389Z</t>
+  </si>
+  <si>
+    <t>About — WKND Adventures</t>
+  </si>
+  <si>
+    <t>https://wknd-adventures.com/about.html</t>
+  </si>
+  <si>
     <t>adventures.report.json</t>
   </si>
   <si>
     <t>["hero-adventure","columns-feature","tabs-activity","cards-article","cards-index","cards-promo"]</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>adventures</t>
-  </si>
-  <si>
-    <t>success</t>
-  </si>
-  <si>
-    <t>2026-10-06T18:38:26.686Z</t>
+    <t>2026-10-07T11:58:14.475Z</t>
   </si>
   <si>
     <t>Adventures — WKND Adventures</t>
@@ -67,6 +85,60 @@
     <t>https://wknd-adventures.com/adventures.html</t>
   </si>
   <si>
+    <t>basecamp.report.json</t>
+  </si>
+  <si>
+    <t>["hero-adventure","tabs-activity","accordion-faq","ticker"]</t>
+  </si>
+  <si>
+    <t>basecamp</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:58:19.400Z</t>
+  </si>
+  <si>
+    <t>Basecamp — WKND Adventures</t>
+  </si>
+  <si>
+    <t>https://wknd-adventures.com/basecamp.html</t>
+  </si>
+  <si>
+    <t>community.report.json</t>
+  </si>
+  <si>
+    <t>["hero-adventure","columns-feature","columns-feature","cards-article","cards-index","accordion-faq"]</t>
+  </si>
+  <si>
+    <t>community</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:58:24.391Z</t>
+  </si>
+  <si>
+    <t>Community — WKND Adventures</t>
+  </si>
+  <si>
+    <t>https://wknd-adventures.com/community.html</t>
+  </si>
+  <si>
+    <t>destinations.report.json</t>
+  </si>
+  <si>
+    <t>["hero-adventure","columns-feature","cards-article","cards-article","cards-promo"]</t>
+  </si>
+  <si>
+    <t>destinations</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:58:28.585Z</t>
+  </si>
+  <si>
+    <t>Destinations — WKND Adventures</t>
+  </si>
+  <si>
+    <t>https://wknd-adventures.com/destinations.html</t>
+  </si>
+  <si>
     <t>expeditions.report.json</t>
   </si>
   <si>
@@ -76,7 +148,7 @@
     <t>expeditions</t>
   </si>
   <si>
-    <t>2026-10-06T18:38:31.724Z</t>
+    <t>2026-10-07T11:58:33.747Z</t>
   </si>
   <si>
     <t>Expeditions — WKND Adventures</t>
@@ -85,6 +157,78 @@
     <t>https://wknd-adventures.com/expeditions.html</t>
   </si>
   <si>
+    <t>faq.report.json</t>
+  </si>
+  <si>
+    <t>["hero-adventure","cards-article","accordion-faq","accordion-faq","accordion-faq","accordion-faq","accordion-faq"]</t>
+  </si>
+  <si>
+    <t>faq</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:58:38.396Z</t>
+  </si>
+  <si>
+    <t>FAQ — WKND Adventures</t>
+  </si>
+  <si>
+    <t>https://wknd-adventures.com/faq.html</t>
+  </si>
+  <si>
+    <t>field-notes.report.json</t>
+  </si>
+  <si>
+    <t>["hero-adventure","columns-feature","cards-article"]</t>
+  </si>
+  <si>
+    <t>field-notes</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:58:43.072Z</t>
+  </si>
+  <si>
+    <t>Field Notes — WKND Adventures</t>
+  </si>
+  <si>
+    <t>https://wknd-adventures.com/field-notes.html</t>
+  </si>
+  <si>
+    <t>gear.report.json</t>
+  </si>
+  <si>
+    <t>["hero-adventure","columns-feature","tabs-activity","cards-index","cards-promo"]</t>
+  </si>
+  <si>
+    <t>gear</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:58:48.089Z</t>
+  </si>
+  <si>
+    <t>Gear — WKND Adventures</t>
+  </si>
+  <si>
+    <t>https://wknd-adventures.com/gear.html</t>
+  </si>
+  <si>
+    <t>index.report.json</t>
+  </si>
+  <si>
+    <t>["hero-adventure","columns-feature","tabs-activity","cards-index","accordion-faq","ticker","gallery-adventure"]</t>
+  </si>
+  <si>
+    <t>index</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:58:03.641Z</t>
+  </si>
+  <si>
+    <t>WKND Adventures — Bold Stories. Real Life. Wild Places.</t>
+  </si>
+  <si>
+    <t>https://wknd-adventures.com/</t>
+  </si>
+  <si>
     <t>nav.report.json</t>
   </si>
   <si>
@@ -92,6 +236,459 @@
   </si>
   <si>
     <t>2026-10-06T14:11:05.371Z</t>
+  </si>
+  <si>
+    <t>sustainability.report.json</t>
+  </si>
+  <si>
+    <t>["hero-adventure","columns-feature","cards-article","cards-index","cards-promo"]</t>
+  </si>
+  <si>
+    <t>sustainability</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:58:52.881Z</t>
+  </si>
+  <si>
+    <t>Sustainability — WKND Adventures</t>
+  </si>
+  <si>
+    <t>https://wknd-adventures.com/sustainability.html</t>
+  </si>
+  <si>
+    <t>us/en.report.json</t>
+  </si>
+  <si>
+    <t>["carousel-wknd-hero","columns-magazine","cards-magazine","cards-magazine","hero-wknd-teaser"]</t>
+  </si>
+  <si>
+    <t>us/en</t>
+  </si>
+  <si>
+    <t>wknd-site-home</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:17:30.655Z</t>
+  </si>
+  <si>
+    <t>WKND Adventures and Travel</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en.html</t>
+  </si>
+  <si>
+    <t>us/en/about-us.report.json</t>
+  </si>
+  <si>
+    <t>["cards-wknd-contributor","cards-wknd-contributor","cards-wknd-contributor","cards-wknd-contributor","cards-wknd-contributor","cards-wknd-contributor","cards-wknd-contributor"]</t>
+  </si>
+  <si>
+    <t>us/en/about-us</t>
+  </si>
+  <si>
+    <t>wknd-site-about</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:16:44.117Z</t>
+  </si>
+  <si>
+    <t>About Us</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/about-us.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures.report.json</t>
+  </si>
+  <si>
+    <t>["hero-wknd","cards-wknd-adventure"]</t>
+  </si>
+  <si>
+    <t>us/en/adventures</t>
+  </si>
+  <si>
+    <t>wknd-site-adventures</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:16:35.769Z</t>
+  </si>
+  <si>
+    <t>Adventures</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures.html</t>
+  </si>
+  <si>
+    <t>us/en/faqs.report.json</t>
+  </si>
+  <si>
+    <t>["accordion-wknd"]</t>
+  </si>
+  <si>
+    <t>us/en/faqs</t>
+  </si>
+  <si>
+    <t>wknd-site-faqs</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:16:52.394Z</t>
+  </si>
+  <si>
+    <t>FAQs</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/faqs.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine.report.json</t>
+  </si>
+  <si>
+    <t>["columns-magazine","cards-magazine","cards-magazine-secure","cards-magazine-secure"]</t>
+  </si>
+  <si>
+    <t>us/en/magazine</t>
+  </si>
+  <si>
+    <t>magazine</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:16:27.048Z</t>
+  </si>
+  <si>
+    <t>Magazine</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp.report.json</t>
+  </si>
+  <si>
+    <t>["breadcrumb-wknd","carousel-wknd","columns-wknd-details","tabs-wknd"]</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp</t>
+  </si>
+  <si>
+    <t>wknd-site-adventure-detail</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:17:39.278Z</t>
+  </si>
+  <si>
+    <t>Bali Surf Camp</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/bali-surf-camp.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/beervana-portland.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/beervana-portland</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:17:44.338Z</t>
+  </si>
+  <si>
+    <t>Beervana in Portland</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/beervana-portland.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/climbing-new-zealand.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/climbing-new-zealand</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:17:48.853Z</t>
+  </si>
+  <si>
+    <t>Climbing New Zealand</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/climbing-new-zealand.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/colorado-rock-climbing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/colorado-rock-climbing</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:17:52.542Z</t>
+  </si>
+  <si>
+    <t>Colorado Rock Climbing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/colorado-rock-climbing.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-southern-utah.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-southern-utah</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:17:58.488Z</t>
+  </si>
+  <si>
+    <t>Cycling Southern Utah</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/cycling-southern-utah.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-tuscany.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-tuscany</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:18:04.220Z</t>
+  </si>
+  <si>
+    <t>Cycling Tuscany</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/cycling-tuscany.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/downhill-skiing-wyoming.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/downhill-skiing-wyoming</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:18:09.844Z</t>
+  </si>
+  <si>
+    <t>Downhill Skiing Wyoming</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/downhill-skiing-wyoming.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/gastronomic-marais-tour.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/gastronomic-marais-tour</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:18:13.988Z</t>
+  </si>
+  <si>
+    <t>Gastronomic Marais Tour</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/gastronomic-marais-tour.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/napa-wine-tasting.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/napa-wine-tasting</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:18:18.097Z</t>
+  </si>
+  <si>
+    <t>Napa Wine Tasting</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/napa-wine-tasting.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/riverside-camping-australia.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/riverside-camping-australia</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:18:23.283Z</t>
+  </si>
+  <si>
+    <t>Riverside Camping</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/riverside-camping-australia.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/ski-touring-mont-blanc.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/ski-touring-mont-blanc</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:18:28.742Z</t>
+  </si>
+  <si>
+    <t>Ski Touring Mont Blanc</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/ski-touring-mont-blanc.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/surf-camp-costa-rica.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/surf-camp-costa-rica</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:18:33.843Z</t>
+  </si>
+  <si>
+    <t>Surf Camp in Costa Rica</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/surf-camp-costa-rica.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/tahoe-skiing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/tahoe-skiing</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:18:38.243Z</t>
+  </si>
+  <si>
+    <t>Tahoe Skiing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/tahoe-skiing.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/west-coast-cycling.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/west-coast-cycling</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:18:44.415Z</t>
+  </si>
+  <si>
+    <t>West Coast Cycling</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/west-coast-cycling.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/whistler-mountain-biking.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/whistler-mountain-biking</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:18:50.141Z</t>
+  </si>
+  <si>
+    <t>Whistler Mountain Biking</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/whistler-mountain-biking.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/yosemite-backpacking.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/yosemite-backpacking</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:18:55.294Z</t>
+  </si>
+  <si>
+    <t>Yosemite Backpacking</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/yosemite-backpacking.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/arctic-surfing.report.json</t>
+  </si>
+  <si>
+    <t>["breadcrumb-wknd","columns-wknd-author"]</t>
+  </si>
+  <si>
+    <t>us/en/magazine/arctic-surfing</t>
+  </si>
+  <si>
+    <t>wknd-site-article</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:17:00.124Z</t>
+  </si>
+  <si>
+    <t>Arctic Surfing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/arctic-surfing.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/guide-la-skateparks.report.json</t>
+  </si>
+  <si>
+    <t>["breadcrumb-wknd","quote-wknd","columns-wknd-author"]</t>
+  </si>
+  <si>
+    <t>us/en/magazine/guide-la-skateparks</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:17:04.588Z</t>
+  </si>
+  <si>
+    <t>Ultimate Guide to LA Skateparks</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/guide-la-skateparks.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/san-diego-surf.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/san-diego-surf</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:17:10.091Z</t>
+  </si>
+  <si>
+    <t>San Diego Surf Spots</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/san-diego-surf.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/ski-touring.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/ski-touring</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:17:15.374Z</t>
+  </si>
+  <si>
+    <t>Ski Touring</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/ski-touring.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/western-australia.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/western-australia</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:17:21.189Z</t>
+  </si>
+  <si>
+    <t>Western Australia</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/western-australia.html</t>
   </si>
 </sst>
 </file>
@@ -480,18 +1077,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="25" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
+    <col min="1" max="2" width="50" customWidth="1"/>
     <col min="3" max="3" width="7" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="4" max="4" width="46" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="7" max="7" width="28" customWidth="1"/>
     <col min="8" max="8" width="26" customWidth="1"/>
-    <col min="9" max="9" width="31" customWidth="1"/>
-    <col min="10" max="10" width="46" customWidth="1"/>
+    <col min="9" max="10" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -546,30 +1141,30 @@
         <v>14</v>
       </c>
       <c r="G2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
         <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E3" t="s">
         <v>12</v>
@@ -578,7 +1173,7 @@
         <v>14</v>
       </c>
       <c r="G3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H3" t="s">
         <v>21</v>
@@ -595,31 +1190,1151 @@
         <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I5" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" t="s">
+        <v>40</v>
+      </c>
+      <c r="J6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" t="s">
+        <v>45</v>
+      </c>
+      <c r="I7" t="s">
+        <v>46</v>
+      </c>
+      <c r="J7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" t="s">
+        <v>51</v>
+      </c>
+      <c r="I8" t="s">
+        <v>52</v>
+      </c>
+      <c r="J8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" t="s">
+        <v>56</v>
+      </c>
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" t="s">
+        <v>57</v>
+      </c>
+      <c r="I9" t="s">
+        <v>58</v>
+      </c>
+      <c r="J9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" t="s">
+        <v>62</v>
+      </c>
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" t="s">
+        <v>63</v>
+      </c>
+      <c r="I10" t="s">
+        <v>64</v>
+      </c>
+      <c r="J10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" t="s">
+        <v>68</v>
+      </c>
+      <c r="E11" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" t="s">
+        <v>69</v>
+      </c>
+      <c r="I11" t="s">
+        <v>70</v>
+      </c>
+      <c r="J11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12">
         <v>16</v>
       </c>
-      <c r="D4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E4">
+      <c r="D12" t="s">
+        <v>73</v>
+      </c>
+      <c r="E12">
         <v>5</v>
       </c>
-      <c r="F4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I4" t="s">
-        <v>25</v>
-      </c>
-      <c r="J4" t="s">
-        <v>17</v>
+      <c r="F12" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" t="s">
+        <v>12</v>
+      </c>
+      <c r="H12" t="s">
+        <v>74</v>
+      </c>
+      <c r="I12" t="s">
+        <v>73</v>
+      </c>
+      <c r="J12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>75</v>
+      </c>
+      <c r="B13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" t="s">
+        <v>77</v>
+      </c>
+      <c r="E13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" t="s">
+        <v>78</v>
+      </c>
+      <c r="I13" t="s">
+        <v>79</v>
+      </c>
+      <c r="J13" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B14" t="s">
+        <v>82</v>
+      </c>
+      <c r="C14" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" t="s">
+        <v>83</v>
+      </c>
+      <c r="E14" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" t="s">
+        <v>84</v>
+      </c>
+      <c r="H14" t="s">
+        <v>85</v>
+      </c>
+      <c r="I14" t="s">
+        <v>86</v>
+      </c>
+      <c r="J14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>88</v>
+      </c>
+      <c r="B15" t="s">
+        <v>89</v>
+      </c>
+      <c r="C15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" t="s">
+        <v>90</v>
+      </c>
+      <c r="E15" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" t="s">
+        <v>91</v>
+      </c>
+      <c r="H15" t="s">
+        <v>92</v>
+      </c>
+      <c r="I15" t="s">
+        <v>93</v>
+      </c>
+      <c r="J15" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>95</v>
+      </c>
+      <c r="B16" t="s">
+        <v>96</v>
+      </c>
+      <c r="C16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" t="s">
+        <v>97</v>
+      </c>
+      <c r="E16" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" t="s">
+        <v>98</v>
+      </c>
+      <c r="H16" t="s">
+        <v>99</v>
+      </c>
+      <c r="I16" t="s">
+        <v>100</v>
+      </c>
+      <c r="J16" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>102</v>
+      </c>
+      <c r="B17" t="s">
+        <v>103</v>
+      </c>
+      <c r="C17" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" t="s">
+        <v>104</v>
+      </c>
+      <c r="E17" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" t="s">
+        <v>105</v>
+      </c>
+      <c r="H17" t="s">
+        <v>106</v>
+      </c>
+      <c r="I17" t="s">
+        <v>107</v>
+      </c>
+      <c r="J17" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>109</v>
+      </c>
+      <c r="B18" t="s">
+        <v>110</v>
+      </c>
+      <c r="C18" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" t="s">
+        <v>111</v>
+      </c>
+      <c r="E18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" t="s">
+        <v>112</v>
+      </c>
+      <c r="H18" t="s">
+        <v>113</v>
+      </c>
+      <c r="I18" t="s">
+        <v>114</v>
+      </c>
+      <c r="J18" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>116</v>
+      </c>
+      <c r="B19" t="s">
+        <v>117</v>
+      </c>
+      <c r="C19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" t="s">
+        <v>118</v>
+      </c>
+      <c r="E19" t="s">
+        <v>12</v>
+      </c>
+      <c r="F19" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" t="s">
+        <v>119</v>
+      </c>
+      <c r="H19" t="s">
+        <v>120</v>
+      </c>
+      <c r="I19" t="s">
+        <v>121</v>
+      </c>
+      <c r="J19" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>123</v>
+      </c>
+      <c r="B20" t="s">
+        <v>117</v>
+      </c>
+      <c r="C20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" t="s">
+        <v>124</v>
+      </c>
+      <c r="E20" t="s">
+        <v>12</v>
+      </c>
+      <c r="F20" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" t="s">
+        <v>119</v>
+      </c>
+      <c r="H20" t="s">
+        <v>125</v>
+      </c>
+      <c r="I20" t="s">
+        <v>126</v>
+      </c>
+      <c r="J20" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>128</v>
+      </c>
+      <c r="B21" t="s">
+        <v>117</v>
+      </c>
+      <c r="C21" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21" t="s">
+        <v>129</v>
+      </c>
+      <c r="E21" t="s">
+        <v>12</v>
+      </c>
+      <c r="F21" t="s">
+        <v>14</v>
+      </c>
+      <c r="G21" t="s">
+        <v>119</v>
+      </c>
+      <c r="H21" t="s">
+        <v>130</v>
+      </c>
+      <c r="I21" t="s">
+        <v>131</v>
+      </c>
+      <c r="J21" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B22" t="s">
+        <v>117</v>
+      </c>
+      <c r="C22" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" t="s">
+        <v>134</v>
+      </c>
+      <c r="E22" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" t="s">
+        <v>119</v>
+      </c>
+      <c r="H22" t="s">
+        <v>135</v>
+      </c>
+      <c r="I22" t="s">
+        <v>136</v>
+      </c>
+      <c r="J22" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>138</v>
+      </c>
+      <c r="B23" t="s">
+        <v>117</v>
+      </c>
+      <c r="C23" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" t="s">
+        <v>139</v>
+      </c>
+      <c r="E23" t="s">
+        <v>12</v>
+      </c>
+      <c r="F23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G23" t="s">
+        <v>119</v>
+      </c>
+      <c r="H23" t="s">
+        <v>140</v>
+      </c>
+      <c r="I23" t="s">
+        <v>141</v>
+      </c>
+      <c r="J23" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>143</v>
+      </c>
+      <c r="B24" t="s">
+        <v>117</v>
+      </c>
+      <c r="C24" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" t="s">
+        <v>144</v>
+      </c>
+      <c r="E24" t="s">
+        <v>12</v>
+      </c>
+      <c r="F24" t="s">
+        <v>14</v>
+      </c>
+      <c r="G24" t="s">
+        <v>119</v>
+      </c>
+      <c r="H24" t="s">
+        <v>145</v>
+      </c>
+      <c r="I24" t="s">
+        <v>146</v>
+      </c>
+      <c r="J24" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>148</v>
+      </c>
+      <c r="B25" t="s">
+        <v>117</v>
+      </c>
+      <c r="C25" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" t="s">
+        <v>149</v>
+      </c>
+      <c r="E25" t="s">
+        <v>12</v>
+      </c>
+      <c r="F25" t="s">
+        <v>14</v>
+      </c>
+      <c r="G25" t="s">
+        <v>119</v>
+      </c>
+      <c r="H25" t="s">
+        <v>150</v>
+      </c>
+      <c r="I25" t="s">
+        <v>151</v>
+      </c>
+      <c r="J25" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>153</v>
+      </c>
+      <c r="B26" t="s">
+        <v>117</v>
+      </c>
+      <c r="C26" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" t="s">
+        <v>154</v>
+      </c>
+      <c r="E26" t="s">
+        <v>12</v>
+      </c>
+      <c r="F26" t="s">
+        <v>14</v>
+      </c>
+      <c r="G26" t="s">
+        <v>119</v>
+      </c>
+      <c r="H26" t="s">
+        <v>155</v>
+      </c>
+      <c r="I26" t="s">
+        <v>156</v>
+      </c>
+      <c r="J26" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>158</v>
+      </c>
+      <c r="B27" t="s">
+        <v>117</v>
+      </c>
+      <c r="C27" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" t="s">
+        <v>159</v>
+      </c>
+      <c r="E27" t="s">
+        <v>12</v>
+      </c>
+      <c r="F27" t="s">
+        <v>14</v>
+      </c>
+      <c r="G27" t="s">
+        <v>119</v>
+      </c>
+      <c r="H27" t="s">
+        <v>160</v>
+      </c>
+      <c r="I27" t="s">
+        <v>161</v>
+      </c>
+      <c r="J27" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>163</v>
+      </c>
+      <c r="B28" t="s">
+        <v>117</v>
+      </c>
+      <c r="C28" t="s">
+        <v>12</v>
+      </c>
+      <c r="D28" t="s">
+        <v>164</v>
+      </c>
+      <c r="E28" t="s">
+        <v>12</v>
+      </c>
+      <c r="F28" t="s">
+        <v>14</v>
+      </c>
+      <c r="G28" t="s">
+        <v>119</v>
+      </c>
+      <c r="H28" t="s">
+        <v>165</v>
+      </c>
+      <c r="I28" t="s">
+        <v>166</v>
+      </c>
+      <c r="J28" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>168</v>
+      </c>
+      <c r="B29" t="s">
+        <v>117</v>
+      </c>
+      <c r="C29" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" t="s">
+        <v>169</v>
+      </c>
+      <c r="E29" t="s">
+        <v>12</v>
+      </c>
+      <c r="F29" t="s">
+        <v>14</v>
+      </c>
+      <c r="G29" t="s">
+        <v>119</v>
+      </c>
+      <c r="H29" t="s">
+        <v>170</v>
+      </c>
+      <c r="I29" t="s">
+        <v>171</v>
+      </c>
+      <c r="J29" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>173</v>
+      </c>
+      <c r="B30" t="s">
+        <v>117</v>
+      </c>
+      <c r="C30" t="s">
+        <v>12</v>
+      </c>
+      <c r="D30" t="s">
+        <v>174</v>
+      </c>
+      <c r="E30" t="s">
+        <v>12</v>
+      </c>
+      <c r="F30" t="s">
+        <v>14</v>
+      </c>
+      <c r="G30" t="s">
+        <v>119</v>
+      </c>
+      <c r="H30" t="s">
+        <v>175</v>
+      </c>
+      <c r="I30" t="s">
+        <v>176</v>
+      </c>
+      <c r="J30" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>178</v>
+      </c>
+      <c r="B31" t="s">
+        <v>117</v>
+      </c>
+      <c r="C31" t="s">
+        <v>12</v>
+      </c>
+      <c r="D31" t="s">
+        <v>179</v>
+      </c>
+      <c r="E31" t="s">
+        <v>12</v>
+      </c>
+      <c r="F31" t="s">
+        <v>14</v>
+      </c>
+      <c r="G31" t="s">
+        <v>119</v>
+      </c>
+      <c r="H31" t="s">
+        <v>180</v>
+      </c>
+      <c r="I31" t="s">
+        <v>181</v>
+      </c>
+      <c r="J31" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>183</v>
+      </c>
+      <c r="B32" t="s">
+        <v>117</v>
+      </c>
+      <c r="C32" t="s">
+        <v>12</v>
+      </c>
+      <c r="D32" t="s">
+        <v>184</v>
+      </c>
+      <c r="E32" t="s">
+        <v>12</v>
+      </c>
+      <c r="F32" t="s">
+        <v>14</v>
+      </c>
+      <c r="G32" t="s">
+        <v>119</v>
+      </c>
+      <c r="H32" t="s">
+        <v>185</v>
+      </c>
+      <c r="I32" t="s">
+        <v>186</v>
+      </c>
+      <c r="J32" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>188</v>
+      </c>
+      <c r="B33" t="s">
+        <v>117</v>
+      </c>
+      <c r="C33" t="s">
+        <v>12</v>
+      </c>
+      <c r="D33" t="s">
+        <v>189</v>
+      </c>
+      <c r="E33" t="s">
+        <v>12</v>
+      </c>
+      <c r="F33" t="s">
+        <v>14</v>
+      </c>
+      <c r="G33" t="s">
+        <v>119</v>
+      </c>
+      <c r="H33" t="s">
+        <v>190</v>
+      </c>
+      <c r="I33" t="s">
+        <v>191</v>
+      </c>
+      <c r="J33" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>193</v>
+      </c>
+      <c r="B34" t="s">
+        <v>117</v>
+      </c>
+      <c r="C34" t="s">
+        <v>12</v>
+      </c>
+      <c r="D34" t="s">
+        <v>194</v>
+      </c>
+      <c r="E34" t="s">
+        <v>12</v>
+      </c>
+      <c r="F34" t="s">
+        <v>14</v>
+      </c>
+      <c r="G34" t="s">
+        <v>119</v>
+      </c>
+      <c r="H34" t="s">
+        <v>195</v>
+      </c>
+      <c r="I34" t="s">
+        <v>196</v>
+      </c>
+      <c r="J34" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>198</v>
+      </c>
+      <c r="B35" t="s">
+        <v>199</v>
+      </c>
+      <c r="C35" t="s">
+        <v>12</v>
+      </c>
+      <c r="D35" t="s">
+        <v>200</v>
+      </c>
+      <c r="E35" t="s">
+        <v>12</v>
+      </c>
+      <c r="F35" t="s">
+        <v>14</v>
+      </c>
+      <c r="G35" t="s">
+        <v>201</v>
+      </c>
+      <c r="H35" t="s">
+        <v>202</v>
+      </c>
+      <c r="I35" t="s">
+        <v>203</v>
+      </c>
+      <c r="J35" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>205</v>
+      </c>
+      <c r="B36" t="s">
+        <v>206</v>
+      </c>
+      <c r="C36" t="s">
+        <v>12</v>
+      </c>
+      <c r="D36" t="s">
+        <v>207</v>
+      </c>
+      <c r="E36" t="s">
+        <v>12</v>
+      </c>
+      <c r="F36" t="s">
+        <v>14</v>
+      </c>
+      <c r="G36" t="s">
+        <v>201</v>
+      </c>
+      <c r="H36" t="s">
+        <v>208</v>
+      </c>
+      <c r="I36" t="s">
+        <v>209</v>
+      </c>
+      <c r="J36" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>211</v>
+      </c>
+      <c r="B37" t="s">
+        <v>199</v>
+      </c>
+      <c r="C37" t="s">
+        <v>12</v>
+      </c>
+      <c r="D37" t="s">
+        <v>212</v>
+      </c>
+      <c r="E37" t="s">
+        <v>12</v>
+      </c>
+      <c r="F37" t="s">
+        <v>14</v>
+      </c>
+      <c r="G37" t="s">
+        <v>201</v>
+      </c>
+      <c r="H37" t="s">
+        <v>213</v>
+      </c>
+      <c r="I37" t="s">
+        <v>214</v>
+      </c>
+      <c r="J37" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>216</v>
+      </c>
+      <c r="B38" t="s">
+        <v>206</v>
+      </c>
+      <c r="C38" t="s">
+        <v>12</v>
+      </c>
+      <c r="D38" t="s">
+        <v>217</v>
+      </c>
+      <c r="E38" t="s">
+        <v>12</v>
+      </c>
+      <c r="F38" t="s">
+        <v>14</v>
+      </c>
+      <c r="G38" t="s">
+        <v>201</v>
+      </c>
+      <c r="H38" t="s">
+        <v>218</v>
+      </c>
+      <c r="I38" t="s">
+        <v>219</v>
+      </c>
+      <c r="J38" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>221</v>
+      </c>
+      <c r="B39" t="s">
+        <v>206</v>
+      </c>
+      <c r="C39" t="s">
+        <v>12</v>
+      </c>
+      <c r="D39" t="s">
+        <v>222</v>
+      </c>
+      <c r="E39" t="s">
+        <v>12</v>
+      </c>
+      <c r="F39" t="s">
+        <v>14</v>
+      </c>
+      <c r="G39" t="s">
+        <v>201</v>
+      </c>
+      <c r="H39" t="s">
+        <v>223</v>
+      </c>
+      <c r="I39" t="s">
+        <v>224</v>
+      </c>
+      <c r="J39" t="s">
+        <v>225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>